<commit_message>
completed entire common error with complaince sheet for priavte as well
</commit_message>
<xml_diff>
--- a/automation_engine/modules/aoc4/excel/Annual Filing common error Output.xlsx
+++ b/automation_engine/modules/aoc4/excel/Annual Filing common error Output.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d6c9e8928e28eb49/process/Tech automation/sample data to arca/Use case/Common Error/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="34" documentId="8_{0328319B-2162-4ED8-9617-BA31723EA9A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC910494-8C73-4852-90E8-8887232F60BD}"/>
+  <xr:revisionPtr revIDLastSave="109" documentId="8_{0328319B-2162-4ED8-9617-BA31723EA9A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{590ABBFB-72B4-47E1-AE4A-86AAA4F9F86D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{5EA3D7FF-880D-4C8A-8F45-837263668CD1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{5EA3D7FF-880D-4C8A-8F45-837263668CD1}"/>
   </bookViews>
   <sheets>
     <sheet name="Common Error" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="compliance sheet for public" sheetId="3" r:id="rId3"/>
     <sheet name="RPT and loans to Director" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="182">
   <si>
     <t>S.No</t>
   </si>
@@ -200,10 +200,22 @@
     <t>Is it a Small Company?</t>
   </si>
   <si>
+    <t>CARO</t>
+  </si>
+  <si>
+    <t>Rotation of Auditors</t>
+  </si>
+  <si>
     <t>IND AS applicability</t>
   </si>
   <si>
     <t>XBRL filing</t>
+  </si>
+  <si>
+    <t>Vigil Mechanism</t>
+  </si>
+  <si>
+    <t>Internal Financial Controls</t>
   </si>
   <si>
     <t>Internal Audit</t>
@@ -240,6 +252,9 @@
     <t>RPT Resolution for omnibus approval</t>
   </si>
   <si>
+    <t>Corporate Social Responsibility</t>
+  </si>
+  <si>
     <t>CSR Committee</t>
   </si>
   <si>
@@ -258,25 +273,37 @@
     <t>Ben 2</t>
   </si>
   <si>
-    <t>CARO</t>
-  </si>
-  <si>
-    <t>Rotation of Auditors</t>
-  </si>
-  <si>
-    <t>Vigil Mechanism</t>
-  </si>
-  <si>
-    <t>Internal Financial Controls</t>
-  </si>
-  <si>
-    <t>Corporate Social Responsibility</t>
-  </si>
-  <si>
     <t>MGT 8 Applicability</t>
   </si>
   <si>
     <t>Certification of MGT 7</t>
+  </si>
+  <si>
+    <t>Previous Year (Year 1)</t>
+  </si>
+  <si>
+    <t>Applicability</t>
+  </si>
+  <si>
+    <t>CS appointment</t>
+  </si>
+  <si>
+    <t>KMP appointment</t>
+  </si>
+  <si>
+    <t>Women Director</t>
+  </si>
+  <si>
+    <t>Independent Director</t>
+  </si>
+  <si>
+    <t>Audit Committee</t>
+  </si>
+  <si>
+    <t>Nomination and Remuneration Committee</t>
+  </si>
+  <si>
+    <t>Annual Board Evaluation</t>
   </si>
   <si>
     <t>SECTION 188</t>
@@ -516,62 +543,106 @@
     <t>If exceeding limit, to mention in MGT 8 &amp; prior approval/ratification in next AGM/EGM</t>
   </si>
   <si>
-    <t>Previous Year (Year 1)</t>
-  </si>
-  <si>
-    <t>Applicability</t>
-  </si>
-  <si>
-    <t>No it is not a small company</t>
-  </si>
-  <si>
-    <t>Applicable</t>
-  </si>
-  <si>
-    <t>CS appointment</t>
-  </si>
-  <si>
-    <t>Whether CRA 2 and CRA 4 filed?</t>
-  </si>
-  <si>
-    <t>KMP appointment</t>
-  </si>
-  <si>
-    <t>Women Director</t>
-  </si>
-  <si>
-    <t>Independent Director</t>
-  </si>
-  <si>
-    <t>Audit Committee</t>
-  </si>
-  <si>
-    <t>Nomination and Remuneration Committee</t>
-  </si>
-  <si>
-    <t>Annual Board Evaluation</t>
-  </si>
-  <si>
-    <t>Not Applicable</t>
-  </si>
-  <si>
-    <t>Need not appoint CS</t>
-  </si>
-  <si>
-    <t>Need not appoint KMP</t>
+    <t xml:space="preserve">Name of the Company: </t>
+  </si>
+  <si>
+    <t>Current Year (Year 0)</t>
+  </si>
+  <si>
+    <t>Financial Particulars</t>
+  </si>
+  <si>
+    <t>Rs.</t>
+  </si>
+  <si>
+    <t>in Cr</t>
+  </si>
+  <si>
+    <t>Paidup capital</t>
+  </si>
+  <si>
+    <t>Reserves and Surplus</t>
+  </si>
+  <si>
+    <t>Total Borrowings</t>
+  </si>
+  <si>
+    <t>Loangiven by Company to Directors or Director related entities (assets)</t>
+  </si>
+  <si>
+    <t>Loans given by Company (assets)</t>
+  </si>
+  <si>
+    <t>Investments made by Company (assets)</t>
+  </si>
+  <si>
+    <t>Corporate Guarantees given by Company</t>
+  </si>
+  <si>
+    <t>Loan from Directors or their relatives (Liabilities)</t>
+  </si>
+  <si>
+    <t>Loan from Shareholders (Liabilities)</t>
+  </si>
+  <si>
+    <t>Secured Loan</t>
+  </si>
+  <si>
+    <t>Advance from Customers, Shareholders, Security Deposits (Liabilitys)</t>
+  </si>
+  <si>
+    <t>Dues to MSME</t>
+  </si>
+  <si>
+    <t>Networth</t>
+  </si>
+  <si>
+    <t>Turnover</t>
+  </si>
+  <si>
+    <t>Total Revenue</t>
+  </si>
+  <si>
+    <t>Profit Before Tax</t>
+  </si>
+  <si>
+    <t>ED / WTD - 1 Monthly Remuneration</t>
+  </si>
+  <si>
+    <t>ED / WTD - 2 Monthly Remuneration</t>
+  </si>
+  <si>
+    <t>Exprt</t>
+  </si>
+  <si>
+    <t>ED / WTD - 5 Monthly Remuneration</t>
+  </si>
+  <si>
+    <t>Sitting Fees to Directors</t>
+  </si>
+  <si>
+    <t>Number of Bodies Corporate Shareholder holding more than 10%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the Company a Holding or a Subsidiary Company </t>
+  </si>
+  <si>
+    <t>Is the Company a Holding, Subsidiary or Associate of IND AS applicable Companies</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="6">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="165" formatCode="_ * #,##0.0000_ ;_ * \-#,##0.0000_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="166" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="167" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="168" formatCode="0.000"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -653,8 +724,22 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -667,8 +752,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -700,12 +791,88 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -754,9 +921,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -770,9 +934,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -780,22 +941,65 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Comma" xfId="2" builtinId="3"/>
     <cellStyle name="Comma 2" xfId="1" xr:uid="{A5D39A03-B88C-4E79-9A9A-6D28B1B6A26D}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <font>
         <condense val="0"/>
@@ -1569,12 +1773,12 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C5">
-    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="NO">
+    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",C5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:C18">
-    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="No">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="No">
       <formula>NOT(ISERROR(SEARCH("No",C5)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1584,7 +1788,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47E73452-E6F6-43B1-B928-978D32056DA3}">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A2:E61"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="54.6640625" customWidth="1"/>
@@ -1594,181 +1798,598 @@
     <col min="5" max="5" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B1" t="s">
+    <row r="2" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="36" t="s">
+        <v>153</v>
+      </c>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="38"/>
+    </row>
+    <row r="3" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="39"/>
+      <c r="B3" s="40" t="s">
+        <v>154</v>
+      </c>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40" t="s">
+        <v>74</v>
+      </c>
+      <c r="E3" s="41"/>
+    </row>
+    <row r="4" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="E4" s="43" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="44" t="s">
+        <v>158</v>
+      </c>
+      <c r="B5" s="45"/>
+      <c r="C5" s="46">
+        <f>B5/10000000</f>
+        <v>0</v>
+      </c>
+      <c r="D5" s="47"/>
+      <c r="E5" s="48">
+        <f t="shared" ref="E5:E13" si="0">D5/10000000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="44" t="s">
+        <v>159</v>
+      </c>
+      <c r="B6" s="45"/>
+      <c r="C6" s="46">
+        <f t="shared" ref="C6:C27" si="1">B6/10000000</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="47"/>
+      <c r="E6" s="48">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="44" t="s">
+        <v>160</v>
+      </c>
+      <c r="B7" s="45"/>
+      <c r="C7" s="46">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D7" s="47"/>
+      <c r="E7" s="48">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="44" t="s">
+        <v>161</v>
+      </c>
+      <c r="B8" s="45"/>
+      <c r="C8" s="46">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D8" s="47"/>
+      <c r="E8" s="48">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="44" t="s">
+        <v>162</v>
+      </c>
+      <c r="B9" s="45"/>
+      <c r="C9" s="46">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D9" s="47"/>
+      <c r="E9" s="48">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="44" t="s">
+        <v>163</v>
+      </c>
+      <c r="B10" s="45"/>
+      <c r="C10" s="46">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D10" s="47"/>
+      <c r="E10" s="48">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="44" t="s">
+        <v>164</v>
+      </c>
+      <c r="B11" s="45"/>
+      <c r="C11" s="46">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D11" s="47"/>
+      <c r="E11" s="48">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="49" t="s">
+        <v>165</v>
+      </c>
+      <c r="B12" s="45"/>
+      <c r="C12" s="46">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D12" s="47"/>
+      <c r="E12" s="48">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="49" t="s">
+        <v>166</v>
+      </c>
+      <c r="B13" s="45"/>
+      <c r="C13" s="46">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D13" s="47"/>
+      <c r="E13" s="48">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="49" t="s">
+        <v>167</v>
+      </c>
+      <c r="B14" s="45"/>
+      <c r="C14" s="46">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D14" s="50"/>
+      <c r="E14" s="48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A15" s="44" t="s">
+        <v>168</v>
+      </c>
+      <c r="B15" s="45"/>
+      <c r="C15" s="46">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D15" s="50"/>
+      <c r="E15" s="48">
+        <f t="shared" ref="E15:E26" si="2">D15/10000000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="49" t="s">
+        <v>169</v>
+      </c>
+      <c r="B16" s="51"/>
+      <c r="C16" s="46">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D16" s="50"/>
+      <c r="E16" s="48">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="52" t="s">
+        <v>170</v>
+      </c>
+      <c r="B17" s="45">
+        <f>+B5+B6</f>
+        <v>0</v>
+      </c>
+      <c r="C17" s="46">
+        <f>B17/10000000</f>
+        <v>0</v>
+      </c>
+      <c r="D17" s="47">
+        <f>+D5+D6</f>
+        <v>0</v>
+      </c>
+      <c r="E17" s="48">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="44" t="s">
+        <v>171</v>
+      </c>
+      <c r="B18" s="45"/>
+      <c r="C18" s="46">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D18" s="47"/>
+      <c r="E18" s="48">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="44" t="s">
+        <v>172</v>
+      </c>
+      <c r="B19" s="45"/>
+      <c r="C19" s="46">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D19" s="47"/>
+      <c r="E19" s="48">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A20" s="44" t="s">
+        <v>173</v>
+      </c>
+      <c r="B20" s="45"/>
+      <c r="C20" s="46">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D20" s="47"/>
+      <c r="E20" s="48">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A21" s="53" t="s">
+        <v>174</v>
+      </c>
+      <c r="B21" s="54"/>
+      <c r="C21" s="8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D21" s="4"/>
+      <c r="E21" s="55">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A22" s="53" t="s">
+        <v>175</v>
+      </c>
+      <c r="B22" s="56"/>
+      <c r="C22" s="8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D22" s="4"/>
+      <c r="E22" s="55">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A23" s="53" t="s">
+        <v>176</v>
+      </c>
+      <c r="B23" s="56"/>
+      <c r="C23" s="8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D23" s="4"/>
+      <c r="E23" s="55">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A24" s="53" t="s">
+        <v>176</v>
+      </c>
+      <c r="B24" s="56"/>
+      <c r="C24" s="8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D24" s="4"/>
+      <c r="E24" s="55">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="53" t="s">
+        <v>177</v>
+      </c>
+      <c r="B25" s="56"/>
+      <c r="C25" s="8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D25" s="4"/>
+      <c r="E25" s="55">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="53" t="s">
+        <v>178</v>
+      </c>
+      <c r="B26" s="56"/>
+      <c r="C26" s="8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D26" s="4"/>
+      <c r="E26" s="55">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A27" s="49" t="s">
+        <v>179</v>
+      </c>
+      <c r="B27" s="51"/>
+      <c r="C27" s="46">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D27" s="4"/>
+      <c r="E27" s="48">
+        <f>D27/10000000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="53" t="s">
+        <v>180</v>
+      </c>
+      <c r="B28" s="57"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="55"/>
+    </row>
+    <row r="29" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A29" s="37" t="s">
+        <v>181</v>
+      </c>
+      <c r="B29" s="37"/>
+      <c r="C29" s="38"/>
+      <c r="D29" s="37"/>
+      <c r="E29" s="38"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B35" t="s">
         <v>43</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D35" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
         <v>45</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C36" t="s">
         <v>46</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E36" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+    <row r="37" spans="1:5" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>59</v>
+      </c>
+      <c r="C49" t="s">
+        <v>60</v>
+      </c>
+      <c r="E49" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>61</v>
+      </c>
+      <c r="C50" t="s">
+        <v>60</v>
+      </c>
+      <c r="E50" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="C57" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="E57" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>55</v>
-      </c>
-      <c r="C15" t="s">
-        <v>56</v>
-      </c>
-      <c r="E15" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>57</v>
-      </c>
-      <c r="C16" t="s">
-        <v>56</v>
-      </c>
-      <c r="E16" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+      <c r="C58" t="s">
+        <v>69</v>
+      </c>
+      <c r="E58" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C23" t="s">
-        <v>64</v>
-      </c>
-      <c r="E23" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>65</v>
-      </c>
-      <c r="C24" t="s">
-        <v>64</v>
-      </c>
-      <c r="E24" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>66</v>
-      </c>
-      <c r="C25" t="s">
-        <v>64</v>
-      </c>
-      <c r="E25" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
+      <c r="C59" t="s">
+        <v>69</v>
+      </c>
+      <c r="E59" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
         <v>73</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="D3:E3"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B28" xr:uid="{EC25BFF7-A12E-4DDB-BFAD-D0F22453AC12}">
+      <formula1>$I$8:$I$10</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B29" xr:uid="{2A1E32FF-253E-4A51-AF04-B5FF416C34A0}">
+      <formula1>$I$6:$I$7</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1778,7 +2399,7 @@
   <dimension ref="A1:F31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="35.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26.5546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="41" customWidth="1"/>
     <col min="5" max="5" width="35.109375" customWidth="1"/>
@@ -1786,30 +2407,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B1" s="34"/>
-      <c r="C1" s="34" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34" t="s">
-        <v>144</v>
-      </c>
-      <c r="F1" s="34"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="F1" s="32"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="32" t="s">
         <v>45</v>
       </c>
-      <c r="C2" s="34" t="s">
-        <v>145</v>
-      </c>
-      <c r="D2" s="34" t="s">
+      <c r="C2" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="D2" s="32" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="34" t="s">
-        <v>145</v>
-      </c>
-      <c r="F2" s="34" t="s">
+      <c r="E2" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="F2" s="32" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1820,25 +2441,13 @@
       <c r="B3" t="s">
         <v>47</v>
       </c>
-      <c r="C3" t="s">
-        <v>146</v>
-      </c>
-      <c r="E3" t="s">
-        <v>146</v>
-      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>67</v>
-      </c>
-      <c r="C4" t="s">
-        <v>147</v>
-      </c>
-      <c r="E4" t="s">
-        <v>147</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -1846,13 +2455,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>68</v>
-      </c>
-      <c r="C5" t="s">
-        <v>156</v>
-      </c>
-      <c r="E5" t="s">
-        <v>156</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -1860,13 +2463,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>49</v>
-      </c>
-      <c r="C6" t="s">
-        <v>156</v>
-      </c>
-      <c r="E6" t="s">
-        <v>147</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -1874,13 +2471,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>69</v>
-      </c>
-      <c r="C7" t="s">
-        <v>156</v>
-      </c>
-      <c r="E7" t="s">
-        <v>156</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -1888,13 +2479,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>70</v>
-      </c>
-      <c r="C8" t="s">
-        <v>147</v>
-      </c>
-      <c r="E8" t="s">
-        <v>147</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -1902,13 +2487,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>50</v>
-      </c>
-      <c r="C9" t="s">
-        <v>156</v>
-      </c>
-      <c r="E9" t="s">
-        <v>156</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -1916,13 +2495,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>51</v>
-      </c>
-      <c r="C10" t="s">
-        <v>156</v>
-      </c>
-      <c r="E10" t="s">
-        <v>156</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -1930,13 +2503,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>148</v>
-      </c>
-      <c r="C11" t="s">
-        <v>157</v>
-      </c>
-      <c r="E11" t="s">
-        <v>157</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -1944,13 +2511,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>53</v>
-      </c>
-      <c r="C12" t="s">
-        <v>156</v>
-      </c>
-      <c r="E12" t="s">
-        <v>156</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -1958,33 +2519,21 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>54</v>
-      </c>
-      <c r="C13" t="s">
-        <v>156</v>
-      </c>
-      <c r="E13" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" s="35" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" s="33" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="33">
         <v>12</v>
       </c>
-      <c r="B14" s="35" t="s">
-        <v>55</v>
-      </c>
-      <c r="C14" s="35" t="s">
-        <v>149</v>
-      </c>
-      <c r="D14" s="35" t="s">
-        <v>56</v>
-      </c>
-      <c r="E14" s="35" t="s">
-        <v>149</v>
-      </c>
-      <c r="F14" s="35" t="s">
-        <v>56</v>
+      <c r="B14" s="33" t="s">
+        <v>59</v>
+      </c>
+      <c r="D14" s="33" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" s="33" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -1992,13 +2541,7 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>58</v>
-      </c>
-      <c r="C15" t="s">
-        <v>156</v>
-      </c>
-      <c r="E15" t="s">
-        <v>156</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -2006,232 +2549,136 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>59</v>
-      </c>
-      <c r="C16" t="s">
-        <v>156</v>
-      </c>
-      <c r="E16" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>60</v>
-      </c>
-      <c r="C17" t="s">
-        <v>156</v>
-      </c>
-      <c r="E17" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>71</v>
-      </c>
-      <c r="C18" t="s">
-        <v>156</v>
-      </c>
-      <c r="E18" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>61</v>
-      </c>
-      <c r="C19" t="s">
-        <v>156</v>
-      </c>
-      <c r="E19" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>62</v>
-      </c>
-      <c r="C20" t="s">
-        <v>156</v>
-      </c>
-      <c r="E20" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>63</v>
-      </c>
-      <c r="C21" t="s">
-        <v>156</v>
+        <v>68</v>
       </c>
       <c r="D21" t="s">
-        <v>64</v>
-      </c>
-      <c r="E21" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>65</v>
-      </c>
-      <c r="C22" t="s">
-        <v>156</v>
+        <v>70</v>
       </c>
       <c r="D22" t="s">
-        <v>64</v>
-      </c>
-      <c r="E22" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>66</v>
-      </c>
-      <c r="C23" t="s">
-        <v>156</v>
+        <v>71</v>
       </c>
       <c r="D23" t="s">
-        <v>64</v>
-      </c>
-      <c r="E23" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>22</v>
       </c>
       <c r="B24" t="s">
         <v>72</v>
       </c>
-      <c r="C24" t="s">
-        <v>156</v>
-      </c>
-      <c r="E24" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>23</v>
       </c>
       <c r="B25" t="s">
         <v>73</v>
       </c>
-      <c r="C25" t="s">
-        <v>147</v>
-      </c>
-      <c r="E25" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>150</v>
-      </c>
-      <c r="C26" t="s">
-        <v>158</v>
-      </c>
-      <c r="E26" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>151</v>
-      </c>
-      <c r="C27" t="s">
-        <v>156</v>
-      </c>
-      <c r="E27" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>152</v>
-      </c>
-      <c r="C28" t="s">
-        <v>156</v>
-      </c>
-      <c r="E28" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>153</v>
-      </c>
-      <c r="C29" t="s">
-        <v>156</v>
-      </c>
-      <c r="E29" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>154</v>
-      </c>
-      <c r="C30" t="s">
-        <v>156</v>
-      </c>
-      <c r="E30" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>155</v>
-      </c>
-      <c r="C31" t="s">
-        <v>156</v>
-      </c>
-      <c r="E31" t="s">
-        <v>156</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -2254,19 +2701,19 @@
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B2" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="2:7" ht="46.8" x14ac:dyDescent="0.3">
       <c r="B4" s="13" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="C4" s="14"/>
       <c r="D4" s="15" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="E4" s="14"/>
       <c r="F4" s="14"/>
@@ -2274,7 +2721,7 @@
     </row>
     <row r="5" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B5" s="13" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="C5" s="14"/>
       <c r="D5" s="14"/>
@@ -2284,7 +2731,7 @@
     </row>
     <row r="6" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B6" s="13" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="C6" s="16"/>
       <c r="D6" s="14"/>
@@ -2294,7 +2741,7 @@
     </row>
     <row r="7" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B7" s="13" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="C7" s="16"/>
       <c r="D7" s="14"/>
@@ -2303,33 +2750,33 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B8" s="32" t="s">
-        <v>81</v>
-      </c>
-      <c r="C8" s="32"/>
-      <c r="D8" s="32"/>
-      <c r="E8" s="32"/>
-      <c r="F8" s="32"/>
-      <c r="G8" s="32"/>
+      <c r="B8" s="34" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
     </row>
     <row r="9" spans="2:7" ht="62.4" x14ac:dyDescent="0.3">
       <c r="B9" s="17" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="F9" s="17" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
     </row>
     <row r="10" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
@@ -2342,13 +2789,13 @@
     </row>
     <row r="11" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B11" s="6" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="E11" s="18">
         <f>+C6</f>
@@ -2359,10 +2806,10 @@
     </row>
     <row r="12" spans="2:7" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B12" s="6" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="D12" s="7"/>
       <c r="E12" s="18">
@@ -2374,10 +2821,10 @@
     </row>
     <row r="13" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B13" s="6" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="D13" s="7"/>
       <c r="E13" s="18">
@@ -2389,10 +2836,10 @@
     </row>
     <row r="14" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B14" s="6" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="D14" s="7"/>
       <c r="E14" s="18">
@@ -2404,10 +2851,10 @@
     </row>
     <row r="15" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B15" s="6" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="D15" s="7"/>
       <c r="E15" s="18">
@@ -2419,10 +2866,10 @@
     </row>
     <row r="16" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B16" s="6" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="D16" s="7"/>
       <c r="E16" s="20">
@@ -2434,10 +2881,10 @@
     </row>
     <row r="17" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B17" s="6" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="D17" s="7"/>
       <c r="E17" s="18">
@@ -2449,10 +2896,10 @@
     </row>
     <row r="18" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B18" s="6" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="D18" s="7"/>
       <c r="E18" s="18">
@@ -2464,10 +2911,10 @@
     </row>
     <row r="19" spans="2:7" ht="28.2" x14ac:dyDescent="0.3">
       <c r="B19" s="21" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="C19" s="21" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="D19" s="7"/>
       <c r="E19" s="22"/>
@@ -2476,10 +2923,10 @@
     </row>
     <row r="20" spans="2:7" ht="28.2" x14ac:dyDescent="0.3">
       <c r="B20" s="21" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="D20" s="7"/>
       <c r="E20" s="22"/>
@@ -2488,52 +2935,52 @@
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B24" s="11" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
     </row>
     <row r="25" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B25" s="23" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="C25" s="24" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="E25" s="17" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
     </row>
     <row r="26" spans="2:7" ht="46.8" x14ac:dyDescent="0.3">
       <c r="B26" s="7" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="D26" s="6"/>
       <c r="E26" s="6"/>
     </row>
     <row r="27" spans="2:7" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B27" s="7" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="D27" s="6"/>
       <c r="E27" s="6"/>
     </row>
     <row r="28" spans="2:7" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B28" s="17" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C28" s="17" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="D28" s="6"/>
       <c r="E28" s="17"/>
@@ -2541,7 +2988,7 @@
     <row r="29" spans="2:7" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B29" s="7"/>
       <c r="C29" s="6" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="D29" s="6"/>
       <c r="E29" s="6"/>
@@ -2549,7 +2996,7 @@
     <row r="30" spans="2:7" ht="46.8" x14ac:dyDescent="0.3">
       <c r="B30" s="7"/>
       <c r="C30" s="6" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="D30" s="17"/>
       <c r="E30" s="6"/>
@@ -2557,157 +3004,157 @@
     <row r="31" spans="2:7" ht="78" x14ac:dyDescent="0.3">
       <c r="B31" s="7"/>
       <c r="C31" s="25" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="D31" s="17"/>
       <c r="E31" s="6"/>
     </row>
     <row r="32" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B32" s="7"/>
-      <c r="C32" s="33" t="s">
-        <v>119</v>
-      </c>
-      <c r="D32" s="33"/>
-      <c r="E32" s="33"/>
+      <c r="C32" s="35" t="s">
+        <v>128</v>
+      </c>
+      <c r="D32" s="35"/>
+      <c r="E32" s="35"/>
     </row>
     <row r="33" spans="2:5" ht="93.6" x14ac:dyDescent="0.3">
       <c r="B33" s="17" t="s">
-        <v>120</v>
-      </c>
-      <c r="C33" s="26" t="s">
-        <v>121</v>
-      </c>
-      <c r="D33" s="26"/>
-      <c r="E33" s="26"/>
+        <v>129</v>
+      </c>
+      <c r="C33" s="31" t="s">
+        <v>130</v>
+      </c>
+      <c r="D33" s="31"/>
+      <c r="E33" s="31"/>
     </row>
     <row r="34" spans="2:5" ht="30.6" x14ac:dyDescent="0.3">
       <c r="B34" s="23" t="s">
-        <v>122</v>
-      </c>
-      <c r="C34" s="27" t="s">
-        <v>123</v>
-      </c>
-      <c r="D34" s="26"/>
-      <c r="E34" s="26"/>
+        <v>131</v>
+      </c>
+      <c r="C34" s="26" t="s">
+        <v>132</v>
+      </c>
+      <c r="D34" s="31"/>
+      <c r="E34" s="31"/>
     </row>
     <row r="35" spans="2:5" ht="31.8" x14ac:dyDescent="0.3">
       <c r="B35" s="6"/>
-      <c r="C35" s="28" t="s">
-        <v>124</v>
-      </c>
-      <c r="D35" s="26"/>
-      <c r="E35" s="26"/>
+      <c r="C35" s="27" t="s">
+        <v>133</v>
+      </c>
+      <c r="D35" s="31"/>
+      <c r="E35" s="31"/>
     </row>
     <row r="36" spans="2:5" ht="42" x14ac:dyDescent="0.3">
       <c r="B36" s="6"/>
-      <c r="C36" s="28" t="s">
-        <v>125</v>
-      </c>
-      <c r="D36" s="26"/>
-      <c r="E36" s="26"/>
+      <c r="C36" s="27" t="s">
+        <v>134</v>
+      </c>
+      <c r="D36" s="31"/>
+      <c r="E36" s="31"/>
     </row>
     <row r="37" spans="2:5" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B37" s="7"/>
-      <c r="C37" s="26" t="s">
-        <v>126</v>
-      </c>
-      <c r="D37" s="26"/>
-      <c r="E37" s="26"/>
+      <c r="C37" s="31" t="s">
+        <v>135</v>
+      </c>
+      <c r="D37" s="31"/>
+      <c r="E37" s="31"/>
     </row>
     <row r="38" spans="2:5" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B38" s="7"/>
       <c r="C38" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="D38" s="26"/>
-      <c r="E38" s="26"/>
+        <v>136</v>
+      </c>
+      <c r="D38" s="31"/>
+      <c r="E38" s="31"/>
     </row>
     <row r="39" spans="2:5" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B39" s="7"/>
       <c r="C39" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="D39" s="26"/>
-      <c r="E39" s="26"/>
+        <v>137</v>
+      </c>
+      <c r="D39" s="31"/>
+      <c r="E39" s="31"/>
     </row>
     <row r="40" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B40" s="7"/>
-      <c r="C40" s="26"/>
-      <c r="D40" s="26"/>
-      <c r="E40" s="26"/>
+      <c r="C40" s="31"/>
+      <c r="D40" s="31"/>
+      <c r="E40" s="31"/>
     </row>
     <row r="41" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B41" s="29" t="s">
-        <v>129</v>
-      </c>
-      <c r="C41" s="26"/>
-      <c r="D41" s="26"/>
-      <c r="E41" s="26"/>
+      <c r="B41" s="28" t="s">
+        <v>138</v>
+      </c>
+      <c r="C41" s="31"/>
+      <c r="D41" s="31"/>
+      <c r="E41" s="31"/>
     </row>
     <row r="42" spans="2:5" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B42" s="7"/>
-      <c r="C42" s="26" t="s">
-        <v>130</v>
-      </c>
-      <c r="D42" s="26"/>
-      <c r="E42" s="26"/>
+      <c r="C42" s="31" t="s">
+        <v>139</v>
+      </c>
+      <c r="D42" s="31"/>
+      <c r="E42" s="31"/>
     </row>
     <row r="43" spans="2:5" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B43" s="7"/>
-      <c r="C43" s="30" t="s">
-        <v>131</v>
-      </c>
-      <c r="D43" s="26"/>
-      <c r="E43" s="26"/>
+      <c r="C43" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="D43" s="31"/>
+      <c r="E43" s="31"/>
     </row>
     <row r="44" spans="2:5" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B44" s="7"/>
-      <c r="C44" s="30" t="s">
-        <v>132</v>
-      </c>
-      <c r="D44" s="26"/>
-      <c r="E44" s="26"/>
+      <c r="C44" s="29" t="s">
+        <v>141</v>
+      </c>
+      <c r="D44" s="31"/>
+      <c r="E44" s="31"/>
     </row>
     <row r="45" spans="2:5" ht="109.2" x14ac:dyDescent="0.3">
       <c r="B45" s="7"/>
-      <c r="C45" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="D45" s="26"/>
-      <c r="E45" s="26"/>
+      <c r="C45" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="D45" s="31"/>
+      <c r="E45" s="31"/>
     </row>
     <row r="46" spans="2:5" ht="78" x14ac:dyDescent="0.3">
       <c r="B46" s="7"/>
-      <c r="C46" s="26" t="s">
-        <v>134</v>
-      </c>
-      <c r="D46" s="26"/>
-      <c r="E46" s="26"/>
+      <c r="C46" s="31" t="s">
+        <v>143</v>
+      </c>
+      <c r="D46" s="31"/>
+      <c r="E46" s="31"/>
     </row>
     <row r="47" spans="2:5" ht="46.8" x14ac:dyDescent="0.3">
       <c r="B47" s="7"/>
-      <c r="C47" s="30" t="s">
-        <v>135</v>
-      </c>
-      <c r="D47" s="26"/>
-      <c r="E47" s="26"/>
+      <c r="C47" s="29" t="s">
+        <v>144</v>
+      </c>
+      <c r="D47" s="31"/>
+      <c r="E47" s="31"/>
     </row>
     <row r="48" spans="2:5" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B48" s="31" t="s">
-        <v>112</v>
+      <c r="B48" s="30" t="s">
+        <v>121</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="D48" s="6"/>
       <c r="E48" s="6"/>
     </row>
     <row r="49" spans="2:5" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B49" s="31" t="s">
-        <v>137</v>
+      <c r="B49" s="30" t="s">
+        <v>146</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="D49" s="6"/>
       <c r="E49" s="6"/>
@@ -2715,7 +3162,7 @@
     <row r="50" spans="2:5" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B50" s="7"/>
       <c r="C50" s="6" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="D50" s="6"/>
       <c r="E50" s="6"/>
@@ -2723,7 +3170,7 @@
     <row r="51" spans="2:5" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B51" s="7"/>
       <c r="C51" s="6" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="D51" s="6"/>
       <c r="E51" s="6"/>
@@ -2731,7 +3178,7 @@
     <row r="52" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B52" s="7"/>
       <c r="C52" s="6" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="D52" s="6"/>
       <c r="E52" s="6"/>
@@ -2739,7 +3186,7 @@
     <row r="53" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B53" s="7"/>
       <c r="C53" s="6" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="D53" s="6"/>
       <c r="E53" s="6"/>
@@ -2747,7 +3194,7 @@
     <row r="54" spans="2:5" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B54" s="7"/>
       <c r="C54" s="6" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="D54" s="6"/>
       <c r="E54" s="6"/>
@@ -2758,7 +3205,7 @@
     <mergeCell ref="C32:E32"/>
   </mergeCells>
   <conditionalFormatting sqref="G11:G20">
-    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Yes">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Yes">
       <formula>NOT(ISERROR(SEARCH("Yes",G11)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>